<commit_message>
chore: Add Name Of Circle row to JMC and WIP bulk upload sample templates
</commit_message>
<xml_diff>
--- a/frontend/public/jmc_bulk_upload_sample.xlsx
+++ b/frontend/public/jmc_bulk_upload_sample.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetData>
     <row r="1">
       <c r="B1" t="str">
@@ -414,376 +414,381 @@
       </c>
     </row>
     <row r="2">
-      <c r="B2" t="str">
-        <v xml:space="preserve">Name Of Division : </v>
-      </c>
-      <c r="D2" t="str">
-        <v>SOLAN</v>
-      </c>
-      <c r="E2" t="str">
-        <v>SOLAN</v>
-      </c>
-      <c r="F2" t="str">
-        <v>SOLAN</v>
+      <c r="A2" t="str">
+        <v>Name Of Circle :</v>
       </c>
     </row>
     <row r="3">
       <c r="B3" t="str">
-        <v xml:space="preserve">Name Of Sub/Division :  </v>
+        <v xml:space="preserve">Name Of Division : </v>
       </c>
       <c r="D3" t="str">
-        <v>ARKI</v>
+        <v>SOLAN</v>
       </c>
       <c r="E3" t="str">
-        <v>ARKI</v>
+        <v>SOLAN</v>
       </c>
       <c r="F3" t="str">
-        <v>KUNIHAR</v>
+        <v>SOLAN</v>
       </c>
     </row>
     <row r="4">
       <c r="B4" t="str">
-        <v xml:space="preserve">Name Of Sub/Station :  </v>
+        <v xml:space="preserve">Name Of Sub/Division :  </v>
       </c>
       <c r="D4" t="str">
-        <v>33/11 KV ARKI</v>
+        <v>ARKI</v>
       </c>
       <c r="E4" t="str">
-        <v>33/11 KV ARKI</v>
+        <v>ARKI</v>
       </c>
       <c r="F4" t="str">
-        <v>33/11 KV KUNIHAR</v>
+        <v>KUNIHAR</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" t="str">
-        <v xml:space="preserve">Name Of Feeder :  </v>
+        <v xml:space="preserve">Name Of Sub/Station :  </v>
       </c>
       <c r="D5" t="str">
-        <v>11 KV FEEDER NO.1</v>
+        <v>33/11 KV ARKI</v>
       </c>
       <c r="E5" t="str">
-        <v>11 KV FEEDER NO.2</v>
+        <v>33/11 KV ARKI</v>
       </c>
       <c r="F5" t="str">
-        <v>11 KV INDUSTRIAL</v>
+        <v>33/11 KV KUNIHAR</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" t="str">
-        <v xml:space="preserve">Location : </v>
+        <v xml:space="preserve">Name Of Feeder :  </v>
       </c>
       <c r="D6" t="str">
-        <v>ARKI TOWN</v>
+        <v>11 KV FEEDER NO.1</v>
       </c>
       <c r="E6" t="str">
-        <v>ARKI BAZAR</v>
+        <v>11 KV FEEDER NO.2</v>
       </c>
       <c r="F6" t="str">
-        <v>KUNIHAR MAIN</v>
+        <v>11 KV INDUSTRIAL</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" t="str">
-        <v xml:space="preserve">Drawing No :  </v>
+        <v xml:space="preserve">Location : </v>
       </c>
       <c r="D7" t="str">
-        <v>101A</v>
+        <v>ARKI TOWN</v>
       </c>
       <c r="E7" t="str">
-        <v>102B</v>
+        <v>ARKI BAZAR</v>
       </c>
       <c r="F7" t="str">
-        <v>203C</v>
+        <v>KUNIHAR MAIN</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" t="str">
+        <v xml:space="preserve">Drawing No :  </v>
+      </c>
+      <c r="D8" t="str">
+        <v>101A</v>
+      </c>
+      <c r="E8" t="str">
+        <v>102B</v>
+      </c>
+      <c r="F8" t="str">
+        <v>203C</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="str">
         <v>Name of Contractor</v>
       </c>
-      <c r="D8" t="str">
+      <c r="D9" t="str">
         <v>Sample Contractor Pvt Ltd</v>
       </c>
-      <c r="E8" t="str">
+      <c r="E9" t="str">
         <v>Sample Contractor Pvt Ltd</v>
       </c>
-      <c r="F8" t="str">
+      <c r="F9" t="str">
         <v>Sample Contractor Pvt Ltd</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="str">
+    <row r="10">
+      <c r="A10" t="str">
         <v>LOA SR.NO.</v>
       </c>
-      <c r="B9" t="str">
+      <c r="B10" t="str">
         <v>Description</v>
       </c>
-      <c r="C9" t="str">
+      <c r="C10" t="str">
         <v>Unit</v>
       </c>
-      <c r="D9" t="str">
+      <c r="D10" t="str">
         <v>JMC</v>
       </c>
-      <c r="E9" t="str">
+      <c r="E10" t="str">
         <v>JMC</v>
       </c>
-      <c r="F9" t="str">
+      <c r="F10" t="str">
         <v>JMC</v>
       </c>
     </row>
-    <row r="10">
-      <c r="B10" t="str">
+    <row r="11">
+      <c r="B11" t="str">
         <v>AB Cabling works ,33KV,22KV,11KV &amp; LT Line overhead Line Ab Cabling &amp; other Cabling Works</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11">
-        <v>1</v>
-      </c>
-      <c r="B11" t="str">
-        <v>AB Cabling works, 33KV, 22KV, 11KV &amp; LT Line overhead</v>
-      </c>
-      <c r="C11" t="str">
-        <v/>
-      </c>
-      <c r="D11">
-        <v>53</v>
-      </c>
-      <c r="E11">
-        <v>54</v>
-      </c>
-      <c r="F11">
-        <v>27</v>
       </c>
     </row>
     <row r="12">
       <c r="A12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B12" t="str">
-        <v>LT AB Cable on poles [Size: (3x95 Sq. mm) +70sqmm +16 sqmm]</v>
+        <v>AB Cabling works, 33KV, 22KV, 11KV &amp; LT Line overhead</v>
       </c>
       <c r="C12" t="str">
-        <v>km</v>
+        <v/>
       </c>
       <c r="D12">
-        <v>6</v>
+        <v>53</v>
       </c>
       <c r="E12">
-        <v>8</v>
+        <v>54</v>
       </c>
       <c r="F12">
-        <v>14</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13">
       <c r="A13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B13" t="str">
-        <v>Steel Tubular Poles (9 m, Working Load &gt; 200 kgf/m²)</v>
+        <v>LT AB Cable on poles [Size: (3x95 Sq. mm) +70sqmm +16 sqmm]</v>
       </c>
       <c r="C13" t="str">
-        <v>No</v>
+        <v>km</v>
       </c>
       <c r="D13">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E13">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="F13">
-        <v>32</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14">
       <c r="A14">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B14" t="str">
-        <v>Muffs with concrete filling</v>
+        <v>Steel Tubular Poles (9 m, Working Load &gt; 200 kgf/m²)</v>
       </c>
       <c r="C14" t="str">
         <v>No</v>
       </c>
       <c r="D14">
-        <v>44</v>
+        <v>9</v>
       </c>
       <c r="E14">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="F14">
-        <v>6</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15">
       <c r="A15">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B15" t="str">
-        <v>Stay Set Complete</v>
+        <v>Muffs with concrete filling</v>
       </c>
       <c r="C15" t="str">
         <v>No</v>
       </c>
       <c r="D15">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E15">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="F15">
-        <v>40</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16">
       <c r="A16">
+        <v>5</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Stay Set Complete</v>
+      </c>
+      <c r="C16" t="str">
+        <v>No</v>
+      </c>
+      <c r="D16">
+        <v>42</v>
+      </c>
+      <c r="E16">
+        <v>35</v>
+      </c>
+      <c r="F16">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
         <v>6</v>
       </c>
-      <c r="B16" t="str">
+      <c r="B17" t="str">
         <v>Stay Wire (7/3.15 mm) (7.0 kg Per Stay Set)</v>
       </c>
-      <c r="C16" t="str">
+      <c r="C17" t="str">
         <v>Kg</v>
       </c>
-      <c r="D16">
+      <c r="D17">
         <v>51</v>
       </c>
-      <c r="E16">
+      <c r="E17">
         <v>37</v>
       </c>
-      <c r="F16">
+      <c r="F17">
         <v>33</v>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" t="str">
-        <v>HT AB Cable works, 11 KV</v>
-      </c>
-    </row>
     <row r="18">
-      <c r="A18">
-        <v>7</v>
-      </c>
       <c r="B18" t="str">
         <v>HT AB Cable works, 11 KV</v>
       </c>
-      <c r="C18" t="str">
-        <v/>
-      </c>
-      <c r="D18">
-        <v>12</v>
-      </c>
-      <c r="E18">
-        <v>16</v>
-      </c>
-      <c r="F18">
-        <v>54</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B19" t="str">
-        <v>11 KV HT AB Cable [Size: 3x95 Sq. mm]</v>
+        <v>HT AB Cable works, 11 KV</v>
       </c>
       <c r="C19" t="str">
-        <v>km</v>
+        <v/>
       </c>
       <c r="D19">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="E19">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="F19">
-        <v>8</v>
+        <v>54</v>
       </c>
     </row>
     <row r="20">
       <c r="A20">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B20" t="str">
-        <v>HT Poles (11 m, Working Load &gt; 300 kgf/m²)</v>
+        <v>11 KV HT AB Cable [Size: 3x95 Sq. mm]</v>
       </c>
       <c r="C20" t="str">
-        <v>No</v>
+        <v>km</v>
       </c>
       <c r="D20">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="E20">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="F20">
-        <v>20</v>
+        <v>8</v>
       </c>
     </row>
     <row r="21">
       <c r="A21">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B21" t="str">
-        <v>Disc Insulator (11 KV)</v>
+        <v>HT Poles (11 m, Working Load &gt; 300 kgf/m²)</v>
       </c>
       <c r="C21" t="str">
         <v>No</v>
       </c>
       <c r="D21">
-        <v>51</v>
+        <v>25</v>
       </c>
       <c r="E21">
-        <v>7</v>
+        <v>47</v>
       </c>
       <c r="F21">
-        <v>51</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22">
       <c r="A22">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B22" t="str">
-        <v>Lightning Arrester (9 KV, 5 KA)</v>
+        <v>Disc Insulator (11 KV)</v>
       </c>
       <c r="C22" t="str">
         <v>No</v>
       </c>
       <c r="D22">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="E22">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="F22">
-        <v>28</v>
+        <v>51</v>
       </c>
     </row>
     <row r="23">
       <c r="A23">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B23" t="str">
-        <v>DO Fuse Set (11 KV, 100A)</v>
+        <v>Lightning Arrester (9 KV, 5 KA)</v>
       </c>
       <c r="C23" t="str">
         <v>No</v>
       </c>
       <c r="D23">
+        <v>16</v>
+      </c>
+      <c r="E23">
+        <v>28</v>
+      </c>
+      <c r="F23">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <v>12</v>
+      </c>
+      <c r="B24" t="str">
+        <v>DO Fuse Set (11 KV, 100A)</v>
+      </c>
+      <c r="C24" t="str">
+        <v>No</v>
+      </c>
+      <c r="D24">
         <v>53</v>
       </c>
-      <c r="E23">
+      <c r="E24">
         <v>44</v>
       </c>
-      <c r="F23">
+      <c r="F24">
         <v>29</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F24"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>